<commit_message>
optimization model and new functional
</commit_message>
<xml_diff>
--- a/src/main/resources/reports/apk_17.xlsx
+++ b/src/main/resources/reports/apk_17.xlsx
@@ -461,16 +461,16 @@
     <t xml:space="preserve">171240</t>
   </si>
   <si>
-    <t xml:space="preserve">${fertilizerDispenser.atStartDateCount + sprayer.atStartDateCount}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${fertilizerDispenser.incomingCount + sprayer.incomingCount}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${fertilizerDispenser.decommissionedCount + sprayer.decommissionedCount}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${fertilizerDispenser.atEndDateCount + sprayer.atEndDateCount}</t>
+    <t xml:space="preserve">${fertilizer_dispenser.atStartDateCount + sprayer.atStartDateCount}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${fertilizer_dispenser.incomingCount + sprayer.incomingCount}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${fertilizer_dispenser.decommissionedCount + sprayer.decommissionedCount}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${fertilizer_dispenser.atEndDateCount + sprayer.atEndDateCount}</t>
   </si>
   <si>
     <t xml:space="preserve">машины сельскохозяйственные для обработки почвы прочие</t>
@@ -487,7 +487,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${</t>
+      <t xml:space="preserve">${rolling_rinks</t>
     </r>
     <r>
       <rPr>
@@ -497,7 +497,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">rollingRinks.atStartDateCount</t>
+      <t xml:space="preserve">.atStartDateCount</t>
     </r>
     <r>
       <rPr>
@@ -519,7 +519,7 @@
         <family val="1"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${</t>
+      <t xml:space="preserve">${rolling_rinks</t>
     </r>
     <r>
       <rPr>
@@ -529,7 +529,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">rollingRinks.</t>
+      <t xml:space="preserve">.</t>
     </r>
     <r>
       <rPr>
@@ -561,7 +561,7 @@
         <family val="1"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${</t>
+      <t xml:space="preserve">${rolling_rinks</t>
     </r>
     <r>
       <rPr>
@@ -571,7 +571,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">rollingRinks.</t>
+      <t xml:space="preserve">.</t>
     </r>
     <r>
       <rPr>
@@ -603,7 +603,7 @@
         <family val="1"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${</t>
+      <t xml:space="preserve">${rolling_rinks</t>
     </r>
     <r>
       <rPr>
@@ -613,7 +613,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">rollingRinks.</t>
+      <t xml:space="preserve">.</t>
     </r>
     <r>
       <rPr>
@@ -669,7 +669,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">hayHarvester.atStartDateCount</t>
+      <t xml:space="preserve">hay_harvester.atStartDateCount</t>
     </r>
     <r>
       <rPr>
@@ -691,7 +691,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${hayHarvester.</t>
+      <t xml:space="preserve">${hay_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -723,7 +723,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${hayHarvester.</t>
+      <t xml:space="preserve">${hay_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -755,7 +755,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">${hayHarvester.</t>
+      <t xml:space="preserve">${hay_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -819,7 +819,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${combine.</t>
+      <t xml:space="preserve">${combine_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -851,7 +851,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${combine.</t>
+      <t xml:space="preserve">${combine_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -883,7 +883,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${combine.</t>
+      <t xml:space="preserve">${combine_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -915,7 +915,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${combine.</t>
+      <t xml:space="preserve">${combine_harvester.</t>
     </r>
     <r>
       <rPr>
@@ -1314,7 +1314,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">irrigationSystem.atStartDateCount</t>
+      <t xml:space="preserve">irrigation_system.atStartDateCount</t>
     </r>
     <r>
       <rPr>
@@ -1338,7 +1338,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${irrigationSystem</t>
+      <t xml:space="preserve">${irrigation_system</t>
     </r>
     <r>
       <rPr>
@@ -1383,7 +1383,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${irrigationSystem</t>
+      <t xml:space="preserve">${irrigation_system</t>
     </r>
     <r>
       <rPr>
@@ -1407,7 +1407,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">${irrigationSystem</t>
+      <t xml:space="preserve">${irrigation_system</t>
     </r>
     <r>
       <rPr>
@@ -1480,8 +1480,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">${</t>
@@ -1492,6 +1492,7 @@
         <color rgb="FF000000"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">expense_current_period_</t>
     </r>
@@ -1499,8 +1500,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">172130.totalAmount}</t>
@@ -1523,6 +1524,7 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">totalAmount</t>
     </r>
@@ -1530,9 +1532,9 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
-        <charset val="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
       </rPr>
       <t xml:space="preserve">}</t>
     </r>
@@ -1555,8 +1557,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">${</t>
@@ -1567,6 +1569,7 @@
         <color rgb="FF000000"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">expense_current_period_</t>
     </r>
@@ -1574,8 +1577,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">172141.</t>
@@ -1586,6 +1589,7 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">totalAmount</t>
     </r>
@@ -1593,8 +1597,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">}</t>
@@ -1617,18 +1621,9 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">totalAmount</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">}</t>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">totalAmount}</t>
     </r>
   </si>
   <si>
@@ -1661,8 +1656,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">${</t>
@@ -1673,6 +1668,7 @@
         <color rgb="FF000000"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">expense_current_period_</t>
     </r>
@@ -1680,8 +1676,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">172151.</t>
@@ -1692,6 +1688,7 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">totalAmount</t>
     </r>
@@ -1699,8 +1696,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">}</t>
@@ -1723,45 +1720,36 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">totalAmount</t>
-    </r>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">totalAmount}</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">172151.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">172151.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Объем потребляемых нефтепродуктов всех видов - всего</t>
+  </si>
+  <si>
+    <t xml:space="preserve">172160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">тонн</t>
+  </si>
+  <si>
+    <t xml:space="preserve">172161</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">}</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">172151.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">172151.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Объем потребляемых нефтепродуктов всех видов - всего</t>
-  </si>
-  <si>
-    <t xml:space="preserve">172160</t>
-  </si>
-  <si>
-    <t xml:space="preserve">тонн</t>
-  </si>
-  <si>
-    <t xml:space="preserve">172161</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">${</t>
@@ -1772,6 +1760,7 @@
         <color rgb="FF000000"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">expense_current_period_</t>
     </r>
@@ -1779,8 +1768,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">172161.</t>
@@ -1791,6 +1780,7 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">totalAmount</t>
     </r>
@@ -1798,8 +1788,8 @@
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">}</t>
@@ -1822,18 +1812,9 @@
         <color rgb="FF000000"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">totalAmount</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val=""/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">}</t>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">totalAmount}</t>
     </r>
   </si>
   <si>
@@ -1847,14 +1828,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="[=0]\-;General"/>
     <numFmt numFmtId="167" formatCode="@"/>
     <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="169" formatCode="General"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1997,19 +1979,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val=""/>
-      <family val="1"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -2021,6 +1990,7 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2390,19 +2360,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="21" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2422,15 +2392,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="4" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3016,23 +2986,23 @@
       </c>
       <c r="C19" s="37" t="str">
         <f aca="false">C20</f>
-        <v>${combine.atStartDateCount}</v>
+        <v>${combine_harvester.atStartDateCount}</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="38" t="str">
         <f aca="false">E20</f>
-        <v>${combine.incomingCount}</v>
+        <v>${combine_harvester.incomingCount}</v>
       </c>
       <c r="F19" s="15"/>
       <c r="G19" s="15"/>
       <c r="H19" s="38" t="str">
         <f aca="false">H20</f>
-        <v>${combine.decommissionedCount}</v>
+        <v>${combine_harvester.decommissionedCount}</v>
       </c>
       <c r="I19" s="15"/>
       <c r="J19" s="37" t="str">
         <f aca="false">J20</f>
-        <v>${combine.atEndDateCount}</v>
+        <v>${combine_harvester.atEndDateCount}</v>
       </c>
       <c r="K19" s="15"/>
       <c r="L19" s="17"/>
@@ -3385,7 +3355,7 @@
       <c r="K37" s="22"/>
       <c r="L37" s="25"/>
     </row>
-    <row r="38" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
         <v>132</v>
       </c>

</xml_diff>